<commit_message>
fix: major update to add error bar in organelle protein mass fraction
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/mitochondrion_fraction_under_different_input.xlsx
+++ b/data/sce_compartment_curation/mitochondrion_fraction_under_different_input.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:JQ18"/>
+  <dimension ref="A1:JQ20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7665,829 +7665,829 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.1504943012703779</v>
+        <v>0.1376557445904809</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1498367121790855</v>
+        <v>0.137057279053458</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1511565879959165</v>
+        <v>0.1384662516351319</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2150583406635818</v>
+        <v>0.1677370745988023</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2231620140321902</v>
+        <v>0.1749586902014152</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2236545669060883</v>
+        <v>0.1701130376068873</v>
       </c>
       <c r="I9" t="n">
-        <v>0.26244123131678</v>
+        <v>0.2349581643442209</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2632860933902115</v>
+        <v>0.2361676048897264</v>
       </c>
       <c r="K9" t="n">
-        <v>0.2611679855670248</v>
+        <v>0.2328137740211273</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1601274747730506</v>
+        <v>0.1493240368410525</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2445566208950099</v>
+        <v>0.2298295780095723</v>
       </c>
       <c r="N9" t="n">
-        <v>0.2463632757971991</v>
+        <v>0.232240037836941</v>
       </c>
       <c r="O9" t="n">
-        <v>0.2554926979984498</v>
+        <v>0.240656249445181</v>
       </c>
       <c r="P9" t="n">
-        <v>0.2466069199360642</v>
+        <v>0.2348546401305292</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.24701017954402</v>
+        <v>0.2357512404060125</v>
       </c>
       <c r="R9" t="n">
-        <v>0.2387649380428772</v>
+        <v>0.225453737393728</v>
       </c>
       <c r="S9" t="n">
-        <v>0.2556523759457448</v>
+        <v>0.2363772356588056</v>
       </c>
       <c r="T9" t="n">
-        <v>0.2539404329951057</v>
+        <v>0.2366837585950451</v>
       </c>
       <c r="U9" t="n">
-        <v>0.2399104559964693</v>
+        <v>0.2236023115327958</v>
       </c>
       <c r="V9" t="n">
-        <v>0.2636104887129154</v>
+        <v>0.2431374673149801</v>
       </c>
       <c r="W9" t="n">
-        <v>0.267752012391375</v>
+        <v>0.2467924378895049</v>
       </c>
       <c r="X9" t="n">
-        <v>0.268081798649476</v>
+        <v>0.2470712742567638</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.2618434769545236</v>
+        <v>0.2415129478898648</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.2612648906289686</v>
+        <v>0.2418130783592171</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.272534095751618</v>
+        <v>0.2511085335702837</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.231003104356781</v>
+        <v>0.2144313267350408</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.231122829514797</v>
+        <v>0.2145195225121859</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.2196438994846648</v>
+        <v>0.2018062564713866</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.2074268703450586</v>
+        <v>0.1915230356625129</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.2027413126270735</v>
+        <v>0.1877351598079752</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.2128302597815022</v>
+        <v>0.1962039083231177</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.2443728064958518</v>
+        <v>0.232617991748835</v>
       </c>
       <c r="AI9" t="n">
-        <v>0.2420831109720043</v>
+        <v>0.2302445763625759</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.2450668003044725</v>
+        <v>0.2317139669386007</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.2587066974967464</v>
+        <v>0.2440097756101718</v>
       </c>
       <c r="AL9" t="n">
-        <v>0.2525724018776557</v>
+        <v>0.2368743045981012</v>
       </c>
       <c r="AM9" t="n">
-        <v>0.2553367351512791</v>
+        <v>0.2416821836052286</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.2759627487085742</v>
+        <v>0.2579098067650405</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.275846352057135</v>
+        <v>0.257839766568788</v>
       </c>
       <c r="AP9" t="n">
-        <v>0.2762721139284097</v>
+        <v>0.2590936182854472</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0.3111871928487418</v>
+        <v>0.2974782260302849</v>
       </c>
       <c r="AR9" t="n">
-        <v>0.312473659668222</v>
+        <v>0.2985856458651374</v>
       </c>
       <c r="AS9" t="n">
-        <v>0.3155640896522094</v>
+        <v>0.3000204764921959</v>
       </c>
       <c r="AT9" t="n">
-        <v>0.2761821332415807</v>
+        <v>0.2593829680635482</v>
       </c>
       <c r="AU9" t="n">
-        <v>0.2857677908758464</v>
+        <v>0.2681727206450896</v>
       </c>
       <c r="AV9" t="n">
-        <v>0.281824212093991</v>
+        <v>0.262624731916444</v>
       </c>
       <c r="AW9" t="n">
-        <v>0.2585441114118042</v>
+        <v>0.2436269110163431</v>
       </c>
       <c r="AX9" t="n">
-        <v>0.257703326076287</v>
+        <v>0.2434976105888088</v>
       </c>
       <c r="AY9" t="n">
-        <v>0.2412444360682812</v>
+        <v>0.2260838029474705</v>
       </c>
       <c r="AZ9" t="n">
-        <v>0.2475046688337775</v>
+        <v>0.2308679874548037</v>
       </c>
       <c r="BA9" t="n">
-        <v>0.258298064352285</v>
+        <v>0.2410007631062784</v>
       </c>
       <c r="BB9" t="n">
-        <v>0.2512181795946933</v>
+        <v>0.2326222552229568</v>
       </c>
       <c r="BC9" t="n">
-        <v>0.3309740616022826</v>
+        <v>0.3273246206099766</v>
       </c>
       <c r="BD9" t="n">
-        <v>0.2021740315861296</v>
+        <v>0.197464576558903</v>
       </c>
       <c r="BE9" t="n">
-        <v>0.2006421009915974</v>
+        <v>0.1958804136278955</v>
       </c>
       <c r="BF9" t="n">
-        <v>0.2083367003536621</v>
+        <v>0.2037310725064343</v>
       </c>
       <c r="BG9" t="n">
-        <v>0.2091991056709259</v>
+        <v>0.204584704913558</v>
       </c>
       <c r="BH9" t="n">
-        <v>0.1840134648589174</v>
+        <v>0.1778012617592887</v>
       </c>
       <c r="BI9" t="n">
-        <v>0.1848708842328037</v>
+        <v>0.1792878374571227</v>
       </c>
       <c r="BJ9" t="n">
-        <v>0.1860500413127027</v>
+        <v>0.180115994415606</v>
       </c>
       <c r="BK9" t="n">
-        <v>0.1860460491114304</v>
+        <v>0.1806921336702038</v>
       </c>
       <c r="BL9" t="n">
-        <v>0.1890512999279007</v>
+        <v>0.1832974594998562</v>
       </c>
       <c r="BM9" t="n">
-        <v>0.1876861812829415</v>
+        <v>0.1819912452397951</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.2918694885553688</v>
+        <v>0.290035386173167</v>
       </c>
       <c r="BO9" t="n">
-        <v>0.2513173226224832</v>
+        <v>0.2498884829382327</v>
       </c>
       <c r="BP9" t="n">
-        <v>0.2733513941984213</v>
+        <v>0.271371070051709</v>
       </c>
       <c r="BQ9" t="n">
-        <v>0.240030369779968</v>
+        <v>0.2387789117402267</v>
       </c>
       <c r="BR9" t="n">
-        <v>0.2599872649102197</v>
+        <v>0.2577370288975714</v>
       </c>
       <c r="BS9" t="n">
-        <v>0.2538422575847783</v>
+        <v>0.2523565152601103</v>
       </c>
       <c r="BT9" t="n">
-        <v>0.2736799313693495</v>
+        <v>0.27187498226588</v>
       </c>
       <c r="BU9" t="n">
-        <v>0.2683616107669056</v>
+        <v>0.2653198053014467</v>
       </c>
       <c r="BV9" t="n">
-        <v>0.3207070232039196</v>
+        <v>0.3193979104984761</v>
       </c>
       <c r="BW9" t="n">
-        <v>0.3587418328509749</v>
+        <v>0.3571717760844208</v>
       </c>
       <c r="BX9" t="n">
-        <v>0.3749235618357113</v>
+        <v>0.3737422849637534</v>
       </c>
       <c r="BY9" t="n">
-        <v>0.3229257675058441</v>
+        <v>0.3215996656860531</v>
       </c>
       <c r="BZ9" t="n">
-        <v>0.3182549187069435</v>
+        <v>0.3168861734007258</v>
       </c>
       <c r="CA9" t="n">
-        <v>0.3154560873494817</v>
+        <v>0.3141166039936318</v>
       </c>
       <c r="CB9" t="n">
-        <v>0.3242474715766217</v>
+        <v>0.3229970294463078</v>
       </c>
       <c r="CC9" t="n">
-        <v>0.3094150724279993</v>
+        <v>0.3078980564383277</v>
       </c>
       <c r="CD9" t="n">
-        <v>0.3151346581901705</v>
+        <v>0.31360640663336</v>
       </c>
       <c r="CE9" t="n">
-        <v>0.2399740498045858</v>
+        <v>0.2386915661650334</v>
       </c>
       <c r="CF9" t="n">
-        <v>0.3879898130591335</v>
+        <v>0.3852318667836895</v>
       </c>
       <c r="CG9" t="n">
-        <v>0.4196366550421359</v>
+        <v>0.415829345860486</v>
       </c>
       <c r="CH9" t="n">
-        <v>0.1893776446439211</v>
+        <v>0.1839516440509976</v>
       </c>
       <c r="CI9" t="n">
-        <v>0.2041811932323797</v>
+        <v>0.1977033278620338</v>
       </c>
       <c r="CJ9" t="n">
-        <v>0.4203358135664217</v>
+        <v>0.4165219983314235</v>
       </c>
       <c r="CK9" t="n">
-        <v>0.4043246518660522</v>
+        <v>0.4010087647329091</v>
       </c>
       <c r="CL9" t="n">
-        <v>0.5040548455096957</v>
+        <v>0.5007633582547191</v>
       </c>
       <c r="CM9" t="n">
-        <v>0.3805247664890965</v>
+        <v>0.3768053851614644</v>
       </c>
       <c r="CN9" t="n">
-        <v>0.4294656315081642</v>
+        <v>0.424558545571639</v>
       </c>
       <c r="CO9" t="n">
-        <v>0.2191262695092671</v>
+        <v>0.2137894147693507</v>
       </c>
       <c r="CP9" t="n">
-        <v>0.269644069026453</v>
+        <v>0.2638024938044919</v>
       </c>
       <c r="CQ9" t="n">
-        <v>0.2855638385579625</v>
+        <v>0.2800221247872735</v>
       </c>
       <c r="CR9" t="n">
-        <v>0.2799096004120598</v>
+        <v>0.2743631596370864</v>
       </c>
       <c r="CS9" t="n">
-        <v>0.2833650380544029</v>
+        <v>0.2779522004023132</v>
       </c>
       <c r="CT9" t="n">
-        <v>0.2882870976260978</v>
+        <v>0.281132223545144</v>
       </c>
       <c r="CU9" t="n">
-        <v>0.2956822638907292</v>
+        <v>0.2892034929624912</v>
       </c>
       <c r="CV9" t="n">
-        <v>0.2926890871980916</v>
+        <v>0.2861847602750099</v>
       </c>
       <c r="CW9" t="n">
-        <v>0.3071346106289131</v>
+        <v>0.2995321735175028</v>
       </c>
       <c r="CX9" t="n">
-        <v>0.3096511138370671</v>
+        <v>0.3019056867611425</v>
       </c>
       <c r="CY9" t="n">
-        <v>0.3058881709492625</v>
+        <v>0.2988180360926074</v>
       </c>
       <c r="CZ9" t="n">
-        <v>0.3094655732556728</v>
+        <v>0.3033386766354719</v>
       </c>
       <c r="DA9" t="n">
-        <v>0.3136515231192183</v>
+        <v>0.3061500870341841</v>
       </c>
       <c r="DB9" t="n">
-        <v>0.3118276415331958</v>
+        <v>0.3048680455935668</v>
       </c>
       <c r="DC9" t="n">
-        <v>0.3189966199448988</v>
+        <v>0.3129305580777051</v>
       </c>
       <c r="DD9" t="n">
-        <v>0.3198315895627443</v>
+        <v>0.3143699499621088</v>
       </c>
       <c r="DE9" t="n">
-        <v>0.3252188394809268</v>
+        <v>0.3192042609387051</v>
       </c>
       <c r="DF9" t="n">
-        <v>0.3249693547218022</v>
+        <v>0.3200636266294331</v>
       </c>
       <c r="DG9" t="n">
-        <v>0.3234957963017535</v>
+        <v>0.3185621869537149</v>
       </c>
       <c r="DH9" t="n">
-        <v>0.3227476327286125</v>
+        <v>0.3176293604333162</v>
       </c>
       <c r="DI9" t="n">
-        <v>0.3198079283635554</v>
+        <v>0.3146403719921673</v>
       </c>
       <c r="DJ9" t="n">
-        <v>0.3172076407822472</v>
+        <v>0.3103732447360093</v>
       </c>
       <c r="DK9" t="n">
-        <v>0.3175624773112525</v>
+        <v>0.3123169636828265</v>
       </c>
       <c r="DL9" t="n">
-        <v>0.3023794408009736</v>
+        <v>0.2952014955415925</v>
       </c>
       <c r="DM9" t="n">
-        <v>0.302002725529404</v>
+        <v>0.2946599456692369</v>
       </c>
       <c r="DN9" t="n">
-        <v>0.2947662041827289</v>
+        <v>0.2878381622454546</v>
       </c>
       <c r="DO9" t="n">
-        <v>0.2880454086060602</v>
+        <v>0.2811515025149721</v>
       </c>
       <c r="DP9" t="n">
-        <v>0.2845284307511901</v>
+        <v>0.2761643310576837</v>
       </c>
       <c r="DQ9" t="n">
-        <v>0.2703387861291588</v>
+        <v>0.2630350414177434</v>
       </c>
       <c r="DR9" t="n">
-        <v>0.1636995630651025</v>
+        <v>0.1579238018025658</v>
       </c>
       <c r="DS9" t="n">
-        <v>0.1635687313873682</v>
+        <v>0.1585375331193234</v>
       </c>
       <c r="DT9" t="n">
-        <v>0.1655839181345599</v>
+        <v>0.159895573035837</v>
       </c>
       <c r="DU9" t="n">
-        <v>0.1658794841452348</v>
+        <v>0.1602707061814307</v>
       </c>
       <c r="DV9" t="n">
-        <v>0.1643518328726343</v>
+        <v>0.1591801693962753</v>
       </c>
       <c r="DW9" t="n">
-        <v>0.1654723306138037</v>
+        <v>0.1596786974668269</v>
       </c>
       <c r="DX9" t="n">
-        <v>0.1632979142762142</v>
+        <v>0.1599709100429048</v>
       </c>
       <c r="DY9" t="n">
-        <v>0.1645032421683591</v>
+        <v>0.1611767715925301</v>
       </c>
       <c r="DZ9" t="n">
-        <v>0.1654967378854935</v>
+        <v>0.1619702807670724</v>
       </c>
       <c r="EA9" t="n">
-        <v>0.1642787818040162</v>
+        <v>0.1608495335504414</v>
       </c>
       <c r="EB9" t="n">
-        <v>0.1633186527027538</v>
+        <v>0.1597680613860124</v>
       </c>
       <c r="EC9" t="n">
-        <v>0.1661226412809651</v>
+        <v>0.1624489796933983</v>
       </c>
       <c r="ED9" t="n">
-        <v>0.1641956922798437</v>
+        <v>0.1599364066319447</v>
       </c>
       <c r="EE9" t="n">
-        <v>0.1662765782563558</v>
+        <v>0.1617541424586678</v>
       </c>
       <c r="EF9" t="n">
-        <v>0.1629707403934417</v>
+        <v>0.1586935456651883</v>
       </c>
       <c r="EG9" t="n">
-        <v>0.1649715133180473</v>
+        <v>0.1602458538168288</v>
       </c>
       <c r="EH9" t="n">
-        <v>0.1655705500509558</v>
+        <v>0.1613145671906341</v>
       </c>
       <c r="EI9" t="n">
-        <v>0.1660070063848909</v>
+        <v>0.1608976541676661</v>
       </c>
       <c r="EJ9" t="n">
-        <v>0.1635730822312488</v>
+        <v>0.1589374571984018</v>
       </c>
       <c r="EK9" t="n">
-        <v>0.1622202518306258</v>
+        <v>0.1575563934138502</v>
       </c>
       <c r="EL9" t="n">
-        <v>0.1620787845715658</v>
+        <v>0.1575345592632927</v>
       </c>
       <c r="EM9" t="n">
-        <v>0.1618895031880863</v>
+        <v>0.1581622619823642</v>
       </c>
       <c r="EN9" t="n">
-        <v>0.1604599961066594</v>
+        <v>0.1567903682745148</v>
       </c>
       <c r="EO9" t="n">
-        <v>0.1610850565645803</v>
+        <v>0.1571880339962688</v>
       </c>
       <c r="EP9" t="n">
-        <v>0.1623847327206576</v>
+        <v>0.1581751015120741</v>
       </c>
       <c r="EQ9" t="n">
-        <v>0.1647908569009825</v>
+        <v>0.1605135194312727</v>
       </c>
       <c r="ER9" t="n">
-        <v>0.1727261475656842</v>
+        <v>0.1679541031779486</v>
       </c>
       <c r="ES9" t="n">
-        <v>0.1634842474595607</v>
+        <v>0.158902948744778</v>
       </c>
       <c r="ET9" t="n">
-        <v>0.1653607848236582</v>
+        <v>0.1610983905541294</v>
       </c>
       <c r="EU9" t="n">
-        <v>0.1666111969074681</v>
+        <v>0.1620815011978293</v>
       </c>
       <c r="EV9" t="n">
-        <v>0.2672673613215105</v>
+        <v>0.2583000701063927</v>
       </c>
       <c r="EW9" t="n">
-        <v>0.2734195031104297</v>
+        <v>0.2641180135331916</v>
       </c>
       <c r="EX9" t="n">
-        <v>0.2366394024802584</v>
+        <v>0.2292385195846813</v>
       </c>
       <c r="EY9" t="n">
-        <v>0.2384120292370232</v>
+        <v>0.232537848538798</v>
       </c>
       <c r="EZ9" t="n">
-        <v>0.2521751559765796</v>
+        <v>0.2434550257965845</v>
       </c>
       <c r="FA9" t="n">
-        <v>0.2581957672693502</v>
+        <v>0.2489268710066249</v>
       </c>
       <c r="FB9" t="n">
-        <v>0.2435176965947941</v>
+        <v>0.2367034605003118</v>
       </c>
       <c r="FC9" t="n">
-        <v>0.2535617851907919</v>
+        <v>0.2468200507743137</v>
       </c>
       <c r="FD9" t="n">
-        <v>0.3165604605847844</v>
+        <v>0.3121465048790852</v>
       </c>
       <c r="FE9" t="n">
-        <v>0.3111743238158435</v>
+        <v>0.3070424741378507</v>
       </c>
       <c r="FF9" t="n">
-        <v>0.3138835509480399</v>
+        <v>0.3095234028089514</v>
       </c>
       <c r="FG9" t="n">
-        <v>0.3130372694964155</v>
+        <v>0.3086663270340414</v>
       </c>
       <c r="FH9" t="n">
-        <v>0.2719142270053335</v>
+        <v>0.2673665005606559</v>
       </c>
       <c r="FI9" t="n">
-        <v>0.2719964922151413</v>
+        <v>0.267414928543205</v>
       </c>
       <c r="FJ9" t="n">
-        <v>0.21456586252441</v>
+        <v>0.2084363927390869</v>
       </c>
       <c r="FK9" t="n">
-        <v>0.214696475652408</v>
+        <v>0.2084786240765228</v>
       </c>
       <c r="FL9" t="n">
-        <v>0.1704121136910865</v>
+        <v>0.1649919065202653</v>
       </c>
       <c r="FM9" t="n">
-        <v>0.171357127337123</v>
+        <v>0.1662491767989464</v>
       </c>
       <c r="FN9" t="n">
-        <v>0.182483669889744</v>
+        <v>0.170196605478569</v>
       </c>
       <c r="FO9" t="n">
-        <v>0.1844094049017123</v>
+        <v>0.1719945245157584</v>
       </c>
       <c r="FP9" t="n">
-        <v>0.179891931262291</v>
+        <v>0.1688458733636962</v>
       </c>
       <c r="FQ9" t="n">
-        <v>0.1785691623893626</v>
+        <v>0.1676118324909684</v>
       </c>
       <c r="FR9" t="n">
-        <v>0.1746778513420723</v>
+        <v>0.163956968151719</v>
       </c>
       <c r="FS9" t="n">
-        <v>0.176690750721558</v>
+        <v>0.165746790375208</v>
       </c>
       <c r="FT9" t="n">
-        <v>0.179324919479967</v>
+        <v>0.1669829698356913</v>
       </c>
       <c r="FU9" t="n">
-        <v>0.1856779644905083</v>
+        <v>0.1731806041401599</v>
       </c>
       <c r="FV9" t="n">
-        <v>0.3338869401219285</v>
+        <v>0.3281533442400405</v>
       </c>
       <c r="FW9" t="n">
-        <v>0.3347228900382666</v>
+        <v>0.3289593424098931</v>
       </c>
       <c r="FX9" t="n">
-        <v>0.3324538147863046</v>
+        <v>0.3263755510527231</v>
       </c>
       <c r="FY9" t="n">
-        <v>0.3318357247885366</v>
+        <v>0.3260379086802774</v>
       </c>
       <c r="FZ9" t="n">
-        <v>0.3363699236308842</v>
+        <v>0.3305579300571125</v>
       </c>
       <c r="GA9" t="n">
-        <v>0.3368384512431778</v>
+        <v>0.3306666209434271</v>
       </c>
       <c r="GB9" t="n">
-        <v>0.3244862449405914</v>
+        <v>0.3182079949865478</v>
       </c>
       <c r="GC9" t="n">
-        <v>0.3241293402251003</v>
+        <v>0.3176145739836184</v>
       </c>
       <c r="GD9" t="n">
-        <v>0.324344873041822</v>
+        <v>0.3178152409170797</v>
       </c>
       <c r="GE9" t="n">
-        <v>0.3233634974686391</v>
+        <v>0.3172511937872801</v>
       </c>
       <c r="GF9" t="n">
-        <v>0.3102178117234446</v>
+        <v>0.3034923874339318</v>
       </c>
       <c r="GG9" t="n">
-        <v>0.3087238263599352</v>
+        <v>0.3027805145658332</v>
       </c>
       <c r="GH9" t="n">
-        <v>0.2994861096778368</v>
+        <v>0.2932364198273038</v>
       </c>
       <c r="GI9" t="n">
-        <v>0.297065936219532</v>
+        <v>0.2908905850717451</v>
       </c>
       <c r="GJ9" t="n">
-        <v>0.1961873916205849</v>
+        <v>0.18731287663218</v>
       </c>
       <c r="GK9" t="n">
-        <v>0.174482320700427</v>
+        <v>0.1688254618892126</v>
       </c>
       <c r="GL9" t="n">
-        <v>0.1931460080978206</v>
+        <v>0.1890425342547693</v>
       </c>
       <c r="GM9" t="n">
-        <v>0.1858616202866902</v>
+        <v>0.1788117323663222</v>
       </c>
       <c r="GN9" t="n">
-        <v>0.1852440183844562</v>
+        <v>0.1741121380114208</v>
       </c>
       <c r="GO9" t="n">
-        <v>0.2037353188235242</v>
+        <v>0.1975822871285973</v>
       </c>
       <c r="GP9" t="n">
-        <v>0.2033707646214976</v>
+        <v>0.1888358189433278</v>
       </c>
       <c r="GQ9" t="n">
-        <v>0.2005865058777857</v>
+        <v>0.1876164954301243</v>
       </c>
       <c r="GR9" t="n">
-        <v>0.1927981987627196</v>
+        <v>0.1817782934831576</v>
       </c>
       <c r="GS9" t="n">
-        <v>0.2543685256112404</v>
+        <v>0.2462914484062413</v>
       </c>
       <c r="GT9" t="n">
-        <v>0.2543517954675891</v>
+        <v>0.2438717020710761</v>
       </c>
       <c r="GU9" t="n">
-        <v>0.2484150102430076</v>
+        <v>0.2366643669018312</v>
       </c>
       <c r="GV9" t="n">
-        <v>0.2400902183887758</v>
+        <v>0.2281352646721036</v>
       </c>
       <c r="GW9" t="n">
-        <v>0.1985799574076401</v>
+        <v>0.1903899869592937</v>
       </c>
       <c r="GX9" t="n">
-        <v>0.2102525899048044</v>
+        <v>0.2016490627765409</v>
       </c>
       <c r="GY9" t="n">
-        <v>0.2094991317763717</v>
+        <v>0.2006397217362338</v>
       </c>
       <c r="GZ9" t="n">
-        <v>0.206117423436865</v>
+        <v>0.1954251439479459</v>
       </c>
       <c r="HA9" t="n">
-        <v>0.2023311407239236</v>
+        <v>0.1870534241702812</v>
       </c>
       <c r="HB9" t="n">
-        <v>0.1943270561929447</v>
+        <v>0.1829718512248202</v>
       </c>
       <c r="HC9" t="n">
-        <v>0.2008206962661402</v>
+        <v>0.1870839278491946</v>
       </c>
       <c r="HD9" t="n">
-        <v>0.207525793389728</v>
+        <v>0.1981218002684054</v>
       </c>
       <c r="HE9" t="n">
-        <v>0.2146347453833712</v>
+        <v>0.2020792531393073</v>
       </c>
       <c r="HF9" t="n">
-        <v>0.2054738710352414</v>
+        <v>0.1991508529466101</v>
       </c>
       <c r="HG9" t="n">
-        <v>0.2084771261691502</v>
+        <v>0.2047398480859824</v>
       </c>
       <c r="HH9" t="n">
         <v>0.1026077177937928</v>
       </c>
       <c r="HI9" t="n">
-        <v>0.2116244700535416</v>
+        <v>0.2082932000982347</v>
       </c>
       <c r="HJ9" t="n">
-        <v>0.1899907239587451</v>
+        <v>0.1828049966180885</v>
       </c>
       <c r="HK9" t="n">
-        <v>0.123689384556227</v>
+        <v>0.1228406019778438</v>
       </c>
       <c r="HL9" t="n">
-        <v>0.3207070232039196</v>
+        <v>0.3193979104984762</v>
       </c>
       <c r="HM9" t="n">
-        <v>0.2509416827250574</v>
+        <v>0.2464629147686922</v>
       </c>
       <c r="HN9" t="n">
-        <v>0.2581473630443211</v>
+        <v>0.2525581700753007</v>
       </c>
       <c r="HO9" t="n">
-        <v>0.2704190174823927</v>
+        <v>0.263936150663968</v>
       </c>
       <c r="HP9" t="n">
-        <v>0.2625219102326473</v>
+        <v>0.2593411991477269</v>
       </c>
       <c r="HQ9" t="n">
-        <v>0.2262372797144864</v>
+        <v>0.2225569387069117</v>
       </c>
       <c r="HR9" t="n">
-        <v>0.2226938415456373</v>
+        <v>0.2211417732803359</v>
       </c>
       <c r="HS9" t="n">
-        <v>0.1860360880657407</v>
+        <v>0.1840867304748065</v>
       </c>
       <c r="HT9" t="n">
-        <v>0.1812596476895596</v>
+        <v>0.1803626975375985</v>
       </c>
       <c r="HU9" t="n">
-        <v>0.1298628526808346</v>
+        <v>0.1292324321675803</v>
       </c>
       <c r="HV9" t="n">
-        <v>0.2710479216568526</v>
+        <v>0.2688404898138629</v>
       </c>
       <c r="HW9" t="n">
-        <v>0.1785607763493831</v>
+        <v>0.1758217835936773</v>
       </c>
       <c r="HX9" t="n">
-        <v>0.1884494900358528</v>
+        <v>0.1858645562050091</v>
       </c>
       <c r="HY9" t="n">
-        <v>0.1863317445255386</v>
+        <v>0.1777107668885592</v>
       </c>
       <c r="HZ9" t="n">
-        <v>0.1773148952678357</v>
+        <v>0.1731407716558473</v>
       </c>
       <c r="IA9" t="n">
-        <v>0.1599183811606324</v>
+        <v>0.1583553968615375</v>
       </c>
       <c r="IB9" t="n">
-        <v>0.2439563550057113</v>
+        <v>0.1872696817716514</v>
       </c>
       <c r="IC9" t="n">
-        <v>0.1812596476895596</v>
+        <v>0.1803626975375985</v>
       </c>
       <c r="ID9" t="n">
-        <v>0.1904304291203774</v>
+        <v>0.1892783641714831</v>
       </c>
       <c r="IE9" t="n">
-        <v>0.1839681345075422</v>
+        <v>0.1831581479498198</v>
       </c>
       <c r="IF9" t="n">
-        <v>0.179017163144695</v>
+        <v>0.1779724634506805</v>
       </c>
       <c r="IG9" t="n">
-        <v>0.1785607763493831</v>
+        <v>0.1758217835936773</v>
       </c>
       <c r="IH9" t="n">
-        <v>0.188761083585836</v>
+        <v>0.1862565501135536</v>
       </c>
       <c r="II9" t="n">
-        <v>0.1986918942415398</v>
+        <v>0.193736712245644</v>
       </c>
       <c r="IJ9" t="n">
-        <v>0.1599183811606324</v>
+        <v>0.1583553968615375</v>
       </c>
       <c r="IK9" t="n">
-        <v>0.1909771746579439</v>
+        <v>0.1894971081353948</v>
       </c>
       <c r="IL9" t="n">
-        <v>0.1315651772562345</v>
+        <v>0.1309343245234323</v>
       </c>
       <c r="IM9" t="n">
-        <v>0.1629895031829399</v>
+        <v>0.1623746665271859</v>
       </c>
       <c r="IN9" t="n">
-        <v>0.1773148952678357</v>
+        <v>0.1731407716558473</v>
       </c>
       <c r="IO9" t="n">
-        <v>0.1684177101608346</v>
+        <v>0.1610345985978086</v>
       </c>
       <c r="IP9" t="n">
-        <v>0.1441194762523341</v>
+        <v>0.1427097718520487</v>
       </c>
       <c r="IQ9" t="n">
-        <v>0.1268486245192769</v>
+        <v>0.1254426555035625</v>
       </c>
       <c r="IR9" t="n">
-        <v>0.1860360880657407</v>
+        <v>0.1840867304748065</v>
       </c>
       <c r="IS9" t="n">
-        <v>0.1778508455902244</v>
+        <v>0.1761623600749278</v>
       </c>
       <c r="IT9" t="n">
-        <v>0.1814248892703759</v>
+        <v>0.179800406673584</v>
       </c>
       <c r="IU9" t="n">
-        <v>0.2423371737746122</v>
+        <v>0.1861819040553887</v>
       </c>
       <c r="IV9" t="n">
-        <v>0.1899876666310458</v>
+        <v>0.1828020571504162</v>
       </c>
       <c r="IW9" t="n">
-        <v>0.2089529849999229</v>
+        <v>0.2059495607571719</v>
       </c>
       <c r="IX9" t="n">
-        <v>0.298428551848076</v>
+        <v>0.2942717718303187</v>
       </c>
       <c r="IY9" t="n">
-        <v>0.3068223013115334</v>
+        <v>0.3037952902533709</v>
       </c>
       <c r="IZ9" t="n">
-        <v>0.1474829067975701</v>
+        <v>0.1405159632529297</v>
       </c>
       <c r="JA9" t="n">
-        <v>0.1526874302480327</v>
+        <v>0.1452450934131874</v>
       </c>
       <c r="JB9" t="n">
-        <v>0.1496490097076676</v>
+        <v>0.1427965703944925</v>
       </c>
       <c r="JC9" t="n">
-        <v>0.1436947189945291</v>
+        <v>0.1364026865404097</v>
       </c>
       <c r="JD9" t="n">
-        <v>0.1670507759300133</v>
+        <v>0.1592408630497486</v>
       </c>
       <c r="JE9" t="n">
-        <v>0.1580142673643255</v>
+        <v>0.150265034014708</v>
       </c>
       <c r="JF9" t="n">
-        <v>0.1583598643687874</v>
+        <v>0.1506862040268921</v>
       </c>
       <c r="JG9" t="n">
-        <v>0.1656835897437152</v>
+        <v>0.1565755103591392</v>
       </c>
       <c r="JH9" t="n">
-        <v>0.1494310708693447</v>
+        <v>0.1414911525517232</v>
       </c>
       <c r="JI9" t="n">
-        <v>0.1585529994764565</v>
+        <v>0.1501476490793612</v>
       </c>
       <c r="JJ9" t="n">
-        <v>0.1533464968275179</v>
+        <v>0.1455138319777365</v>
       </c>
       <c r="JK9" t="n">
-        <v>0.1633852304704849</v>
+        <v>0.1552925271800936</v>
       </c>
       <c r="JL9" t="n">
-        <v>0.1617194245665232</v>
+        <v>0.1536330637311133</v>
       </c>
       <c r="JM9" t="n">
-        <v>0.1627487056793146</v>
+        <v>0.1546812372930131</v>
       </c>
       <c r="JN9" t="n">
-        <v>0.1773032587292789</v>
+        <v>0.1685504873296774</v>
       </c>
       <c r="JO9" t="n">
-        <v>0.1632282368659465</v>
+        <v>0.1535356903842165</v>
       </c>
       <c r="JP9" t="n">
-        <v>0.1790231640927686</v>
+        <v>0.1703517902489897</v>
       </c>
       <c r="JQ9" t="n">
-        <v>0.1643607579388019</v>
+        <v>0.1545967560014103</v>
       </c>
     </row>
     <row r="10">
@@ -16003,6 +16003,1676 @@
       </c>
       <c r="JQ18" t="n">
         <v>0.01123859933728229</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>m_latest</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.05356623021180258</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.05143959379917534</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.05376468716206442</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.07687181360256705</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.08048194224936996</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.07828941806498219</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.1174120708984491</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.1184322340564445</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.1163317012615886</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.05896188653958643</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.1073672760065304</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.1113670226126323</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.1154394363345735</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.1167706890420141</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.1175240578566823</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0.1108606850736538</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0.1053770012397877</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0.1036420127117786</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0.1051857453495312</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.1044536882753545</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.1056546223249917</v>
+      </c>
+      <c r="X19" t="n">
+        <v>0.1090405192390066</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>0.1101107972610466</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>0.1087987899729642</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0.1114202031297968</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0.09776455285682406</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>0.09921846169577501</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>0.0913272866507889</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>0.08573918524140921</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>0.0801892349886512</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0.08771884454061551</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>0.1114300523144106</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>0.1132938745657167</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>0.106455873178423</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0.1229771363462017</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>0.1176686576269183</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>0.1196093270545851</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>0.1211206438846568</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>0.1207618376869156</v>
+      </c>
+      <c r="AP19" t="n">
+        <v>0.1227836743374965</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>0.1658730545650678</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>0.166676308189795</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>0.1668653659892053</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>0.1163025554732443</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>0.1251882202436752</v>
+      </c>
+      <c r="AV19" t="n">
+        <v>0.1250706573037791</v>
+      </c>
+      <c r="AW19" t="n">
+        <v>0.1203712987829325</v>
+      </c>
+      <c r="AX19" t="n">
+        <v>0.1215169642952754</v>
+      </c>
+      <c r="AY19" t="n">
+        <v>0.1113882749528324</v>
+      </c>
+      <c r="AZ19" t="n">
+        <v>0.1125085473707285</v>
+      </c>
+      <c r="BA19" t="n">
+        <v>0.1108959938892685</v>
+      </c>
+      <c r="BB19" t="n">
+        <v>0.1091844279076603</v>
+      </c>
+      <c r="BC19" t="n">
+        <v>0.1711541094818027</v>
+      </c>
+      <c r="BD19" t="n">
+        <v>0.07782768041973745</v>
+      </c>
+      <c r="BE19" t="n">
+        <v>0.07601851000160539</v>
+      </c>
+      <c r="BF19" t="n">
+        <v>0.06893977415135323</v>
+      </c>
+      <c r="BG19" t="n">
+        <v>0.07024380537229331</v>
+      </c>
+      <c r="BH19" t="n">
+        <v>0.06971592190892879</v>
+      </c>
+      <c r="BI19" t="n">
+        <v>0.0695016415278616</v>
+      </c>
+      <c r="BJ19" t="n">
+        <v>0.06998089604691581</v>
+      </c>
+      <c r="BK19" t="n">
+        <v>0.05636874979954243</v>
+      </c>
+      <c r="BL19" t="n">
+        <v>0.0569329822837747</v>
+      </c>
+      <c r="BM19" t="n">
+        <v>0.05808511439443705</v>
+      </c>
+      <c r="BN19" t="n">
+        <v>0.1602860391918968</v>
+      </c>
+      <c r="BO19" t="n">
+        <v>0.1091396797994515</v>
+      </c>
+      <c r="BP19" t="n">
+        <v>0.1395740073412171</v>
+      </c>
+      <c r="BQ19" t="n">
+        <v>0.1000739223739206</v>
+      </c>
+      <c r="BR19" t="n">
+        <v>0.1343176917770544</v>
+      </c>
+      <c r="BS19" t="n">
+        <v>0.1308557223368775</v>
+      </c>
+      <c r="BT19" t="n">
+        <v>0.1433675040628681</v>
+      </c>
+      <c r="BU19" t="n">
+        <v>0.1370812605194777</v>
+      </c>
+      <c r="BV19" t="n">
+        <v>0.2000367987975165</v>
+      </c>
+      <c r="BW19" t="n">
+        <v>0.2242583326623467</v>
+      </c>
+      <c r="BX19" t="n">
+        <v>0.2469192680956512</v>
+      </c>
+      <c r="BY19" t="n">
+        <v>0.2113475392513041</v>
+      </c>
+      <c r="BZ19" t="n">
+        <v>0.2035519504768519</v>
+      </c>
+      <c r="CA19" t="n">
+        <v>0.2008633720397906</v>
+      </c>
+      <c r="CB19" t="n">
+        <v>0.212092147310622</v>
+      </c>
+      <c r="CC19" t="n">
+        <v>0.1960927921405126</v>
+      </c>
+      <c r="CD19" t="n">
+        <v>0.2011845829833974</v>
+      </c>
+      <c r="CE19" t="n">
+        <v>0.1508883827995558</v>
+      </c>
+      <c r="CF19" t="n">
+        <v>0.2282239523580839</v>
+      </c>
+      <c r="CG19" t="n">
+        <v>0.2580713119387788</v>
+      </c>
+      <c r="CH19" t="n">
+        <v>0.08471906326798145</v>
+      </c>
+      <c r="CI19" t="n">
+        <v>0.09333886288915071</v>
+      </c>
+      <c r="CJ19" t="n">
+        <v>0.2506592169891563</v>
+      </c>
+      <c r="CK19" t="n">
+        <v>0.2500574086779666</v>
+      </c>
+      <c r="CL19" t="n">
+        <v>0.3146094526425441</v>
+      </c>
+      <c r="CM19" t="n">
+        <v>0.2225268614290297</v>
+      </c>
+      <c r="CN19" t="n">
+        <v>0.2573360384488682</v>
+      </c>
+      <c r="CO19" t="n">
+        <v>0.09650340634508506</v>
+      </c>
+      <c r="CP19" t="n">
+        <v>0.1398438309613872</v>
+      </c>
+      <c r="CQ19" t="n">
+        <v>0.1569129125272608</v>
+      </c>
+      <c r="CR19" t="n">
+        <v>0.1518932234288982</v>
+      </c>
+      <c r="CS19" t="n">
+        <v>0.1533284467748268</v>
+      </c>
+      <c r="CT19" t="n">
+        <v>0.1544426217527113</v>
+      </c>
+      <c r="CU19" t="n">
+        <v>0.1615598779994249</v>
+      </c>
+      <c r="CV19" t="n">
+        <v>0.1597486412845009</v>
+      </c>
+      <c r="CW19" t="n">
+        <v>0.1688457701501029</v>
+      </c>
+      <c r="CX19" t="n">
+        <v>0.170548401832527</v>
+      </c>
+      <c r="CY19" t="n">
+        <v>0.1682136929362117</v>
+      </c>
+      <c r="CZ19" t="n">
+        <v>0.1738357797006787</v>
+      </c>
+      <c r="DA19" t="n">
+        <v>0.1738351841547154</v>
+      </c>
+      <c r="DB19" t="n">
+        <v>0.1724281226036775</v>
+      </c>
+      <c r="DC19" t="n">
+        <v>0.1816903895837087</v>
+      </c>
+      <c r="DD19" t="n">
+        <v>0.1841522045263108</v>
+      </c>
+      <c r="DE19" t="n">
+        <v>0.1853783858132388</v>
+      </c>
+      <c r="DF19" t="n">
+        <v>0.190583715326921</v>
+      </c>
+      <c r="DG19" t="n">
+        <v>0.1886829653129275</v>
+      </c>
+      <c r="DH19" t="n">
+        <v>0.1877597524199325</v>
+      </c>
+      <c r="DI19" t="n">
+        <v>0.1845515601870678</v>
+      </c>
+      <c r="DJ19" t="n">
+        <v>0.1789535597738834</v>
+      </c>
+      <c r="DK19" t="n">
+        <v>0.1824436658075155</v>
+      </c>
+      <c r="DL19" t="n">
+        <v>0.165852711457893</v>
+      </c>
+      <c r="DM19" t="n">
+        <v>0.1661060318849066</v>
+      </c>
+      <c r="DN19" t="n">
+        <v>0.161855216230671</v>
+      </c>
+      <c r="DO19" t="n">
+        <v>0.156699589392714</v>
+      </c>
+      <c r="DP19" t="n">
+        <v>0.1503680228806774</v>
+      </c>
+      <c r="DQ19" t="n">
+        <v>0.1419261117528803</v>
+      </c>
+      <c r="DR19" t="n">
+        <v>0.06860603994404263</v>
+      </c>
+      <c r="DS19" t="n">
+        <v>0.07152947611094282</v>
+      </c>
+      <c r="DT19" t="n">
+        <v>0.07208648413403126</v>
+      </c>
+      <c r="DU19" t="n">
+        <v>0.07211616053418152</v>
+      </c>
+      <c r="DV19" t="n">
+        <v>0.07135059612657868</v>
+      </c>
+      <c r="DW19" t="n">
+        <v>0.07099527069640463</v>
+      </c>
+      <c r="DX19" t="n">
+        <v>0.07245678927153808</v>
+      </c>
+      <c r="DY19" t="n">
+        <v>0.07411715990444567</v>
+      </c>
+      <c r="DZ19" t="n">
+        <v>0.07361719903144572</v>
+      </c>
+      <c r="EA19" t="n">
+        <v>0.07362167471415275</v>
+      </c>
+      <c r="EB19" t="n">
+        <v>0.07368469641492528</v>
+      </c>
+      <c r="EC19" t="n">
+        <v>0.07340865562384967</v>
+      </c>
+      <c r="ED19" t="n">
+        <v>0.07347091225140434</v>
+      </c>
+      <c r="EE19" t="n">
+        <v>0.07401866198113831</v>
+      </c>
+      <c r="EF19" t="n">
+        <v>0.07312125598693815</v>
+      </c>
+      <c r="EG19" t="n">
+        <v>0.07188201267549943</v>
+      </c>
+      <c r="EH19" t="n">
+        <v>0.07287235177566621</v>
+      </c>
+      <c r="EI19" t="n">
+        <v>0.07333797760831286</v>
+      </c>
+      <c r="EJ19" t="n">
+        <v>0.07313441739248573</v>
+      </c>
+      <c r="EK19" t="n">
+        <v>0.0723643058475799</v>
+      </c>
+      <c r="EL19" t="n">
+        <v>0.07185256786409663</v>
+      </c>
+      <c r="EM19" t="n">
+        <v>0.07305734229361097</v>
+      </c>
+      <c r="EN19" t="n">
+        <v>0.07241831615397844</v>
+      </c>
+      <c r="EO19" t="n">
+        <v>0.07247669197419898</v>
+      </c>
+      <c r="EP19" t="n">
+        <v>0.07277702664743653</v>
+      </c>
+      <c r="EQ19" t="n">
+        <v>0.07454447038727399</v>
+      </c>
+      <c r="ER19" t="n">
+        <v>0.0787256024560004</v>
+      </c>
+      <c r="ES19" t="n">
+        <v>0.07287678068645752</v>
+      </c>
+      <c r="ET19" t="n">
+        <v>0.07323381430160222</v>
+      </c>
+      <c r="EU19" t="n">
+        <v>0.07384732208606973</v>
+      </c>
+      <c r="EV19" t="n">
+        <v>0.1480168043002744</v>
+      </c>
+      <c r="EW19" t="n">
+        <v>0.1447634225519851</v>
+      </c>
+      <c r="EX19" t="n">
+        <v>0.1069985491736407</v>
+      </c>
+      <c r="EY19" t="n">
+        <v>0.1043198621305688</v>
+      </c>
+      <c r="EZ19" t="n">
+        <v>0.118511045342445</v>
+      </c>
+      <c r="FA19" t="n">
+        <v>0.1184633005658743</v>
+      </c>
+      <c r="FB19" t="n">
+        <v>0.1089054816265726</v>
+      </c>
+      <c r="FC19" t="n">
+        <v>0.1114874869160776</v>
+      </c>
+      <c r="FD19" t="n">
+        <v>0.1871399301384602</v>
+      </c>
+      <c r="FE19" t="n">
+        <v>0.1836681133308368</v>
+      </c>
+      <c r="FF19" t="n">
+        <v>0.1899517144520139</v>
+      </c>
+      <c r="FG19" t="n">
+        <v>0.1868986170114699</v>
+      </c>
+      <c r="FH19" t="n">
+        <v>0.1447585084925895</v>
+      </c>
+      <c r="FI19" t="n">
+        <v>0.1457812271894212</v>
+      </c>
+      <c r="FJ19" t="n">
+        <v>0.114248602473203</v>
+      </c>
+      <c r="FK19" t="n">
+        <v>0.1117915535208851</v>
+      </c>
+      <c r="FL19" t="n">
+        <v>0.08262906033800022</v>
+      </c>
+      <c r="FM19" t="n">
+        <v>0.08384044331576757</v>
+      </c>
+      <c r="FN19" t="n">
+        <v>0.07741253688725627</v>
+      </c>
+      <c r="FO19" t="n">
+        <v>0.07805275813024357</v>
+      </c>
+      <c r="FP19" t="n">
+        <v>0.07655105387826262</v>
+      </c>
+      <c r="FQ19" t="n">
+        <v>0.07765136875394109</v>
+      </c>
+      <c r="FR19" t="n">
+        <v>0.07931896601705234</v>
+      </c>
+      <c r="FS19" t="n">
+        <v>0.08064822533712672</v>
+      </c>
+      <c r="FT19" t="n">
+        <v>0.0818831788126401</v>
+      </c>
+      <c r="FU19" t="n">
+        <v>0.08482060580367994</v>
+      </c>
+      <c r="FV19" t="n">
+        <v>0.2030918078163083</v>
+      </c>
+      <c r="FW19" t="n">
+        <v>0.2045809383305653</v>
+      </c>
+      <c r="FX19" t="n">
+        <v>0.2024725394834358</v>
+      </c>
+      <c r="FY19" t="n">
+        <v>0.2020483956784206</v>
+      </c>
+      <c r="FZ19" t="n">
+        <v>0.208296535311683</v>
+      </c>
+      <c r="GA19" t="n">
+        <v>0.2064788503033885</v>
+      </c>
+      <c r="GB19" t="n">
+        <v>0.1898977093630417</v>
+      </c>
+      <c r="GC19" t="n">
+        <v>0.1888480721599355</v>
+      </c>
+      <c r="GD19" t="n">
+        <v>0.1888466479506992</v>
+      </c>
+      <c r="GE19" t="n">
+        <v>0.1887216362916205</v>
+      </c>
+      <c r="GF19" t="n">
+        <v>0.1789078956929099</v>
+      </c>
+      <c r="GG19" t="n">
+        <v>0.1782622598305872</v>
+      </c>
+      <c r="GH19" t="n">
+        <v>0.172070830950173</v>
+      </c>
+      <c r="GI19" t="n">
+        <v>0.1703010761307143</v>
+      </c>
+      <c r="GJ19" t="n">
+        <v>0.08111385960345499</v>
+      </c>
+      <c r="GK19" t="n">
+        <v>0.07031912902853006</v>
+      </c>
+      <c r="GL19" t="n">
+        <v>0.07868850759212583</v>
+      </c>
+      <c r="GM19" t="n">
+        <v>0.07408332918565459</v>
+      </c>
+      <c r="GN19" t="n">
+        <v>0.07413085201189369</v>
+      </c>
+      <c r="GO19" t="n">
+        <v>0.07754683740022864</v>
+      </c>
+      <c r="GP19" t="n">
+        <v>0.07530360520463461</v>
+      </c>
+      <c r="GQ19" t="n">
+        <v>0.0744329234458101</v>
+      </c>
+      <c r="GR19" t="n">
+        <v>0.07437436806709589</v>
+      </c>
+      <c r="GS19" t="n">
+        <v>0.110927658383907</v>
+      </c>
+      <c r="GT19" t="n">
+        <v>0.1085835086674308</v>
+      </c>
+      <c r="GU19" t="n">
+        <v>0.1029868616889635</v>
+      </c>
+      <c r="GV19" t="n">
+        <v>0.09995651005939311</v>
+      </c>
+      <c r="GW19" t="n">
+        <v>0.08935174558669397</v>
+      </c>
+      <c r="GX19" t="n">
+        <v>0.09557067294716651</v>
+      </c>
+      <c r="GY19" t="n">
+        <v>0.09468774769000272</v>
+      </c>
+      <c r="GZ19" t="n">
+        <v>0.09485001799714743</v>
+      </c>
+      <c r="HA19" t="n">
+        <v>0.08221028098897815</v>
+      </c>
+      <c r="HB19" t="n">
+        <v>0.08128976909433773</v>
+      </c>
+      <c r="HC19" t="n">
+        <v>0.08141866222347785</v>
+      </c>
+      <c r="HD19" t="n">
+        <v>0.09617353750220636</v>
+      </c>
+      <c r="HE19" t="n">
+        <v>0.09803528126893957</v>
+      </c>
+      <c r="HF19" t="n">
+        <v>0.08687653776704357</v>
+      </c>
+      <c r="HG19" t="n">
+        <v>0.08339291108153536</v>
+      </c>
+      <c r="HH19" t="n">
+        <v>0.04943828230218295</v>
+      </c>
+      <c r="HI19" t="n">
+        <v>0.09829261366218459</v>
+      </c>
+      <c r="HJ19" t="n">
+        <v>0.06694695750654872</v>
+      </c>
+      <c r="HK19" t="n">
+        <v>0.05979524333721883</v>
+      </c>
+      <c r="HL19" t="n">
+        <v>0.2000367987975165</v>
+      </c>
+      <c r="HM19" t="n">
+        <v>0.09645832449965737</v>
+      </c>
+      <c r="HN19" t="n">
+        <v>0.08584071421049251</v>
+      </c>
+      <c r="HO19" t="n">
+        <v>0.09415346914890411</v>
+      </c>
+      <c r="HP19" t="n">
+        <v>0.09852250097051342</v>
+      </c>
+      <c r="HQ19" t="n">
+        <v>0.1020114567516975</v>
+      </c>
+      <c r="HR19" t="n">
+        <v>0.1036842811080247</v>
+      </c>
+      <c r="HS19" t="n">
+        <v>0.08704712802860731</v>
+      </c>
+      <c r="HT19" t="n">
+        <v>0.07964069668917412</v>
+      </c>
+      <c r="HU19" t="n">
+        <v>0.03048849087931109</v>
+      </c>
+      <c r="HV19" t="n">
+        <v>0.0629157695870492</v>
+      </c>
+      <c r="HW19" t="n">
+        <v>0.08532764513007306</v>
+      </c>
+      <c r="HX19" t="n">
+        <v>0.01597085356593967</v>
+      </c>
+      <c r="HY19" t="n">
+        <v>0.06095181468792544</v>
+      </c>
+      <c r="HZ19" t="n">
+        <v>0.06665346582643719</v>
+      </c>
+      <c r="IA19" t="n">
+        <v>0.05350650019187821</v>
+      </c>
+      <c r="IB19" t="n">
+        <v>0.09347947565847647</v>
+      </c>
+      <c r="IC19" t="n">
+        <v>0.07964069668917412</v>
+      </c>
+      <c r="ID19" t="n">
+        <v>0.08982922642624583</v>
+      </c>
+      <c r="IE19" t="n">
+        <v>0.07958641400965198</v>
+      </c>
+      <c r="IF19" t="n">
+        <v>0.0996215352693183</v>
+      </c>
+      <c r="IG19" t="n">
+        <v>0.08532764513007306</v>
+      </c>
+      <c r="IH19" t="n">
+        <v>0.09291432506778127</v>
+      </c>
+      <c r="II19" t="n">
+        <v>0.09889872485441478</v>
+      </c>
+      <c r="IJ19" t="n">
+        <v>0.05350650019187821</v>
+      </c>
+      <c r="IK19" t="n">
+        <v>0.08238076839656953</v>
+      </c>
+      <c r="IL19" t="n">
+        <v>0.03039853975977596</v>
+      </c>
+      <c r="IM19" t="n">
+        <v>0.03525111085304409</v>
+      </c>
+      <c r="IN19" t="n">
+        <v>0.06665346582643719</v>
+      </c>
+      <c r="IO19" t="n">
+        <v>0.06346479957759578</v>
+      </c>
+      <c r="IP19" t="n">
+        <v>0.05944834287324013</v>
+      </c>
+      <c r="IQ19" t="n">
+        <v>0.05805622170802995</v>
+      </c>
+      <c r="IR19" t="n">
+        <v>0.08704712802860731</v>
+      </c>
+      <c r="IS19" t="n">
+        <v>0.087843233447012</v>
+      </c>
+      <c r="IT19" t="n">
+        <v>0.07587717138828826</v>
+      </c>
+      <c r="IU19" t="n">
+        <v>0.0929455010733771</v>
+      </c>
+      <c r="IV19" t="n">
+        <v>0.06694588281289499</v>
+      </c>
+      <c r="IW19" t="n">
+        <v>0.08265161005039681</v>
+      </c>
+      <c r="IX19" t="n">
+        <v>0.1459100858435101</v>
+      </c>
+      <c r="IY19" t="n">
+        <v>0.1670627728612122</v>
+      </c>
+      <c r="IZ19" t="n">
+        <v>0.0549630929884919</v>
+      </c>
+      <c r="JA19" t="n">
+        <v>0.0578657461531203</v>
+      </c>
+      <c r="JB19" t="n">
+        <v>0.05660196109227767</v>
+      </c>
+      <c r="JC19" t="n">
+        <v>0.05774716582666458</v>
+      </c>
+      <c r="JD19" t="n">
+        <v>0.06587982551515226</v>
+      </c>
+      <c r="JE19" t="n">
+        <v>0.0624666840225134</v>
+      </c>
+      <c r="JF19" t="n">
+        <v>0.06350220017857108</v>
+      </c>
+      <c r="JG19" t="n">
+        <v>0.06627787399789847</v>
+      </c>
+      <c r="JH19" t="n">
+        <v>0.06097482122838399</v>
+      </c>
+      <c r="JI19" t="n">
+        <v>0.06396201557885148</v>
+      </c>
+      <c r="JJ19" t="n">
+        <v>0.06181670538760226</v>
+      </c>
+      <c r="JK19" t="n">
+        <v>0.06998389058161127</v>
+      </c>
+      <c r="JL19" t="n">
+        <v>0.06874715980040731</v>
+      </c>
+      <c r="JM19" t="n">
+        <v>0.0692347349580032</v>
+      </c>
+      <c r="JN19" t="n">
+        <v>0.07363542172442843</v>
+      </c>
+      <c r="JO19" t="n">
+        <v>0.07249129264457817</v>
+      </c>
+      <c r="JP19" t="n">
+        <v>0.07771568521609007</v>
+      </c>
+      <c r="JQ19" t="n">
+        <v>0.07194011700761228</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>m_latest2</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.130524240594326</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.1269467242564441</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.1310295522993126</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.1982109398742925</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.2055353005032338</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.2075815392639861</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.2346078358306525</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.2359953728283662</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.235100358537476</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.1338959522566037</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.2503538164201691</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.2555900148784488</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.2779865830027061</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.255479672064751</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.2597869252407675</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0.2464181498908675</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0.2584807334158569</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0.2569218754910623</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0.2467652680326381</v>
+      </c>
+      <c r="V20" t="n">
+        <v>0.2574817784112065</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0.2620291428746718</v>
+      </c>
+      <c r="X20" t="n">
+        <v>0.2635944565903627</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0.2554620315189299</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0.2558967682189049</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>0.2680300774716454</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0.2249059984136542</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>0.2249418007282598</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>0.2125293874696531</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>0.1987131999384207</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>0.192557626939998</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>0.2034326298202479</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>0.2531580427088062</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>0.2540106903158513</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>0.2473841975620706</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>0.2584718623703343</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>0.249803421994877</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>0.2569369146669646</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>0.2661787335684959</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>0.2701062033920783</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>0.2700068401116097</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>0.295417711431026</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>0.2997566197444678</v>
+      </c>
+      <c r="AS20" t="n">
+        <v>0.2973293690168179</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>0.2725688176713583</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>0.280033127800502</v>
+      </c>
+      <c r="AV20" t="n">
+        <v>0.273058843531058</v>
+      </c>
+      <c r="AW20" t="n">
+        <v>0.2545463373538085</v>
+      </c>
+      <c r="AX20" t="n">
+        <v>0.2566439274065255</v>
+      </c>
+      <c r="AY20" t="n">
+        <v>0.2392904805584583</v>
+      </c>
+      <c r="AZ20" t="n">
+        <v>0.2481401992914211</v>
+      </c>
+      <c r="BA20" t="n">
+        <v>0.2612253008110854</v>
+      </c>
+      <c r="BB20" t="n">
+        <v>0.2454935689999151</v>
+      </c>
+      <c r="BC20" t="n">
+        <v>0.2931886230318569</v>
+      </c>
+      <c r="BD20" t="n">
+        <v>0.1621929219411003</v>
+      </c>
+      <c r="BE20" t="n">
+        <v>0.1572490020049999</v>
+      </c>
+      <c r="BF20" t="n">
+        <v>0.1641078639217959</v>
+      </c>
+      <c r="BG20" t="n">
+        <v>0.1645785284085099</v>
+      </c>
+      <c r="BH20" t="n">
+        <v>0.1394968219714606</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>0.1400800642241599</v>
+      </c>
+      <c r="BJ20" t="n">
+        <v>0.1405218064716135</v>
+      </c>
+      <c r="BK20" t="n">
+        <v>0.1297100414248369</v>
+      </c>
+      <c r="BL20" t="n">
+        <v>0.134883197326191</v>
+      </c>
+      <c r="BM20" t="n">
+        <v>0.1356331699888036</v>
+      </c>
+      <c r="BN20" t="n">
+        <v>0.2776023822017727</v>
+      </c>
+      <c r="BO20" t="n">
+        <v>0.2278305891447364</v>
+      </c>
+      <c r="BP20" t="n">
+        <v>0.2625035087140502</v>
+      </c>
+      <c r="BQ20" t="n">
+        <v>0.2150829516376776</v>
+      </c>
+      <c r="BR20" t="n">
+        <v>0.2227565222545337</v>
+      </c>
+      <c r="BS20" t="n">
+        <v>0.218065884459773</v>
+      </c>
+      <c r="BT20" t="n">
+        <v>0.2351780127241678</v>
+      </c>
+      <c r="BU20" t="n">
+        <v>0.2319930471432197</v>
+      </c>
+      <c r="BV20" t="n">
+        <v>0.3158989655368283</v>
+      </c>
+      <c r="BW20" t="n">
+        <v>0.3347750907735955</v>
+      </c>
+      <c r="BX20" t="n">
+        <v>0.3402048058449779</v>
+      </c>
+      <c r="BY20" t="n">
+        <v>0.295866178309155</v>
+      </c>
+      <c r="BZ20" t="n">
+        <v>0.3132794917093799</v>
+      </c>
+      <c r="CA20" t="n">
+        <v>0.3093482886000781</v>
+      </c>
+      <c r="CB20" t="n">
+        <v>0.3109208611304839</v>
+      </c>
+      <c r="CC20" t="n">
+        <v>0.3094838962080086</v>
+      </c>
+      <c r="CD20" t="n">
+        <v>0.3104853943073985</v>
+      </c>
+      <c r="CE20" t="n">
+        <v>0.2271501437776524</v>
+      </c>
+      <c r="CF20" t="n">
+        <v>0.3598583086354101</v>
+      </c>
+      <c r="CG20" t="n">
+        <v>0.3719407967258229</v>
+      </c>
+      <c r="CH20" t="n">
+        <v>0.1795868860840901</v>
+      </c>
+      <c r="CI20" t="n">
+        <v>0.1912462011169623</v>
+      </c>
+      <c r="CJ20" t="n">
+        <v>0.3799883158233493</v>
+      </c>
+      <c r="CK20" t="n">
+        <v>0.3731983125023277</v>
+      </c>
+      <c r="CL20" t="n">
+        <v>0.430910889360665</v>
+      </c>
+      <c r="CM20" t="n">
+        <v>0.3405388108613616</v>
+      </c>
+      <c r="CN20" t="n">
+        <v>0.3874912640288669</v>
+      </c>
+      <c r="CO20" t="n">
+        <v>0.2083470873908297</v>
+      </c>
+      <c r="CP20" t="n">
+        <v>0.2546761560425586</v>
+      </c>
+      <c r="CQ20" t="n">
+        <v>0.3103136925800925</v>
+      </c>
+      <c r="CR20" t="n">
+        <v>0.3106532523532388</v>
+      </c>
+      <c r="CS20" t="n">
+        <v>0.3097805060053019</v>
+      </c>
+      <c r="CT20" t="n">
+        <v>0.3107937255830881</v>
+      </c>
+      <c r="CU20" t="n">
+        <v>0.3125540324564838</v>
+      </c>
+      <c r="CV20" t="n">
+        <v>0.3152620931341082</v>
+      </c>
+      <c r="CW20" t="n">
+        <v>0.3084230180319551</v>
+      </c>
+      <c r="CX20" t="n">
+        <v>0.3103713273570324</v>
+      </c>
+      <c r="CY20" t="n">
+        <v>0.3085719624781251</v>
+      </c>
+      <c r="CZ20" t="n">
+        <v>0.3025942098540537</v>
+      </c>
+      <c r="DA20" t="n">
+        <v>0.3041573108803169</v>
+      </c>
+      <c r="DB20" t="n">
+        <v>0.3039676591841828</v>
+      </c>
+      <c r="DC20" t="n">
+        <v>0.3032616529011116</v>
+      </c>
+      <c r="DD20" t="n">
+        <v>0.3002807349034602</v>
+      </c>
+      <c r="DE20" t="n">
+        <v>0.3062481528933582</v>
+      </c>
+      <c r="DF20" t="n">
+        <v>0.3009470855132205</v>
+      </c>
+      <c r="DG20" t="n">
+        <v>0.2993695504982691</v>
+      </c>
+      <c r="DH20" t="n">
+        <v>0.299317782459372</v>
+      </c>
+      <c r="DI20" t="n">
+        <v>0.2940084181411317</v>
+      </c>
+      <c r="DJ20" t="n">
+        <v>0.2889373822479187</v>
+      </c>
+      <c r="DK20" t="n">
+        <v>0.2918210323254788</v>
+      </c>
+      <c r="DL20" t="n">
+        <v>0.2744980329276552</v>
+      </c>
+      <c r="DM20" t="n">
+        <v>0.2745494156053079</v>
+      </c>
+      <c r="DN20" t="n">
+        <v>0.2681762425991102</v>
+      </c>
+      <c r="DO20" t="n">
+        <v>0.2616183379705993</v>
+      </c>
+      <c r="DP20" t="n">
+        <v>0.2587074309702222</v>
+      </c>
+      <c r="DQ20" t="n">
+        <v>0.246300627095536</v>
+      </c>
+      <c r="DR20" t="n">
+        <v>0.1376836350356793</v>
+      </c>
+      <c r="DS20" t="n">
+        <v>0.1387756561950488</v>
+      </c>
+      <c r="DT20" t="n">
+        <v>0.1414046637351624</v>
+      </c>
+      <c r="DU20" t="n">
+        <v>0.1414706949359255</v>
+      </c>
+      <c r="DV20" t="n">
+        <v>0.1399135051813876</v>
+      </c>
+      <c r="DW20" t="n">
+        <v>0.1409057017700591</v>
+      </c>
+      <c r="DX20" t="n">
+        <v>0.1357235806656142</v>
+      </c>
+      <c r="DY20" t="n">
+        <v>0.1380115117603828</v>
+      </c>
+      <c r="DZ20" t="n">
+        <v>0.1382549999007045</v>
+      </c>
+      <c r="EA20" t="n">
+        <v>0.137288078095881</v>
+      </c>
+      <c r="EB20" t="n">
+        <v>0.1376565260140481</v>
+      </c>
+      <c r="EC20" t="n">
+        <v>0.1381326061408327</v>
+      </c>
+      <c r="ED20" t="n">
+        <v>0.1379500401136529</v>
+      </c>
+      <c r="EE20" t="n">
+        <v>0.1410235844571939</v>
+      </c>
+      <c r="EF20" t="n">
+        <v>0.1386191958339842</v>
+      </c>
+      <c r="EG20" t="n">
+        <v>0.1384080969875549</v>
+      </c>
+      <c r="EH20" t="n">
+        <v>0.1390695736364076</v>
+      </c>
+      <c r="EI20" t="n">
+        <v>0.1407628227341982</v>
+      </c>
+      <c r="EJ20" t="n">
+        <v>0.1381456772349905</v>
+      </c>
+      <c r="EK20" t="n">
+        <v>0.1370465806684009</v>
+      </c>
+      <c r="EL20" t="n">
+        <v>0.1364263332701048</v>
+      </c>
+      <c r="EM20" t="n">
+        <v>0.1357326401559052</v>
+      </c>
+      <c r="EN20" t="n">
+        <v>0.135363069319851</v>
+      </c>
+      <c r="EO20" t="n">
+        <v>0.1350211480566119</v>
+      </c>
+      <c r="EP20" t="n">
+        <v>0.1377940422820726</v>
+      </c>
+      <c r="EQ20" t="n">
+        <v>0.140231295486842</v>
+      </c>
+      <c r="ER20" t="n">
+        <v>0.1459832527129686</v>
+      </c>
+      <c r="ES20" t="n">
+        <v>0.1377528811045648</v>
+      </c>
+      <c r="ET20" t="n">
+        <v>0.1387607684527666</v>
+      </c>
+      <c r="EU20" t="n">
+        <v>0.1400480762451618</v>
+      </c>
+      <c r="EV20" t="n">
+        <v>0.2562460807344586</v>
+      </c>
+      <c r="EW20" t="n">
+        <v>0.2568057895244195</v>
+      </c>
+      <c r="EX20" t="n">
+        <v>0.221959164553189</v>
+      </c>
+      <c r="EY20" t="n">
+        <v>0.2238998505839307</v>
+      </c>
+      <c r="EZ20" t="n">
+        <v>0.23658522669325</v>
+      </c>
+      <c r="FA20" t="n">
+        <v>0.2399294996312145</v>
+      </c>
+      <c r="FB20" t="n">
+        <v>0.2256637815784265</v>
+      </c>
+      <c r="FC20" t="n">
+        <v>0.2373842343480621</v>
+      </c>
+      <c r="FD20" t="n">
+        <v>0.3361419236616182</v>
+      </c>
+      <c r="FE20" t="n">
+        <v>0.3237833496781867</v>
+      </c>
+      <c r="FF20" t="n">
+        <v>0.3206185174308728</v>
+      </c>
+      <c r="FG20" t="n">
+        <v>0.3218124834170641</v>
+      </c>
+      <c r="FH20" t="n">
+        <v>0.2483974850480592</v>
+      </c>
+      <c r="FI20" t="n">
+        <v>0.2488377573663255</v>
+      </c>
+      <c r="FJ20" t="n">
+        <v>0.2022154988525574</v>
+      </c>
+      <c r="FK20" t="n">
+        <v>0.2017411881210213</v>
+      </c>
+      <c r="FL20" t="n">
+        <v>0.1642338150767818</v>
+      </c>
+      <c r="FM20" t="n">
+        <v>0.1655864779506919</v>
+      </c>
+      <c r="FN20" t="n">
+        <v>0.1691787592728962</v>
+      </c>
+      <c r="FO20" t="n">
+        <v>0.1714816598302983</v>
+      </c>
+      <c r="FP20" t="n">
+        <v>0.1696349867850827</v>
+      </c>
+      <c r="FQ20" t="n">
+        <v>0.1685360379162781</v>
+      </c>
+      <c r="FR20" t="n">
+        <v>0.1670618354691914</v>
+      </c>
+      <c r="FS20" t="n">
+        <v>0.1685640719198004</v>
+      </c>
+      <c r="FT20" t="n">
+        <v>0.173367577238219</v>
+      </c>
+      <c r="FU20" t="n">
+        <v>0.1789644323766945</v>
+      </c>
+      <c r="FV20" t="n">
+        <v>0.3250132753047261</v>
+      </c>
+      <c r="FW20" t="n">
+        <v>0.3249538881429764</v>
+      </c>
+      <c r="FX20" t="n">
+        <v>0.3187992295888023</v>
+      </c>
+      <c r="FY20" t="n">
+        <v>0.3175510543046187</v>
+      </c>
+      <c r="FZ20" t="n">
+        <v>0.3166432162306646</v>
+      </c>
+      <c r="GA20" t="n">
+        <v>0.3144196489921524</v>
+      </c>
+      <c r="GB20" t="n">
+        <v>0.2982277853152508</v>
+      </c>
+      <c r="GC20" t="n">
+        <v>0.2976029481743865</v>
+      </c>
+      <c r="GD20" t="n">
+        <v>0.2977692903941272</v>
+      </c>
+      <c r="GE20" t="n">
+        <v>0.2976460393568858</v>
+      </c>
+      <c r="GF20" t="n">
+        <v>0.28496653340944</v>
+      </c>
+      <c r="GG20" t="n">
+        <v>0.2836442184485876</v>
+      </c>
+      <c r="GH20" t="n">
+        <v>0.2752268944946831</v>
+      </c>
+      <c r="GI20" t="n">
+        <v>0.2735014810238148</v>
+      </c>
+      <c r="GJ20" t="n">
+        <v>0.1831495381794874</v>
+      </c>
+      <c r="GK20" t="n">
+        <v>0.1783174372073257</v>
+      </c>
+      <c r="GL20" t="n">
+        <v>0.1815115357789749</v>
+      </c>
+      <c r="GM20" t="n">
+        <v>0.171814320940419</v>
+      </c>
+      <c r="GN20" t="n">
+        <v>0.1698943509234444</v>
+      </c>
+      <c r="GO20" t="n">
+        <v>0.2004189287454289</v>
+      </c>
+      <c r="GP20" t="n">
+        <v>0.1881962761795289</v>
+      </c>
+      <c r="GQ20" t="n">
+        <v>0.1857947058316254</v>
+      </c>
+      <c r="GR20" t="n">
+        <v>0.1775003416145918</v>
+      </c>
+      <c r="GS20" t="n">
+        <v>0.2426137698907213</v>
+      </c>
+      <c r="GT20" t="n">
+        <v>0.2354801508180152</v>
+      </c>
+      <c r="GU20" t="n">
+        <v>0.2252111323880979</v>
+      </c>
+      <c r="GV20" t="n">
+        <v>0.2172261434876189</v>
+      </c>
+      <c r="GW20" t="n">
+        <v>0.1806309395753564</v>
+      </c>
+      <c r="GX20" t="n">
+        <v>0.1889613295449661</v>
+      </c>
+      <c r="GY20" t="n">
+        <v>0.1890167146925752</v>
+      </c>
+      <c r="GZ20" t="n">
+        <v>0.1893322052224152</v>
+      </c>
+      <c r="HA20" t="n">
+        <v>0.1923329582792733</v>
+      </c>
+      <c r="HB20" t="n">
+        <v>0.1799588089287391</v>
+      </c>
+      <c r="HC20" t="n">
+        <v>0.1868673794871106</v>
+      </c>
+      <c r="HD20" t="n">
+        <v>0.1909800757618199</v>
+      </c>
+      <c r="HE20" t="n">
+        <v>0.1965251035736243</v>
+      </c>
+      <c r="HF20" t="n">
+        <v>0.1887341668729774</v>
+      </c>
+      <c r="HG20" t="n">
+        <v>0.1895384183164869</v>
+      </c>
+      <c r="HH20" t="n">
+        <v>0.1151240408393654</v>
+      </c>
+      <c r="HI20" t="n">
+        <v>0.1998120427920146</v>
+      </c>
+      <c r="HJ20" t="n">
+        <v>0.1738501055230583</v>
+      </c>
+      <c r="HK20" t="n">
+        <v>0.1341379794037464</v>
+      </c>
+      <c r="HL20" t="n">
+        <v>0.3158989655368283</v>
+      </c>
+      <c r="HM20" t="n">
+        <v>0.2345862405275926</v>
+      </c>
+      <c r="HN20" t="n">
+        <v>0.2398276658827735</v>
+      </c>
+      <c r="HO20" t="n">
+        <v>0.251153975127132</v>
+      </c>
+      <c r="HP20" t="n">
+        <v>0.2434843582398767</v>
+      </c>
+      <c r="HQ20" t="n">
+        <v>0.2096536379031325</v>
+      </c>
+      <c r="HR20" t="n">
+        <v>0.2074709879429495</v>
+      </c>
+      <c r="HS20" t="n">
+        <v>0.1787953692988891</v>
+      </c>
+      <c r="HT20" t="n">
+        <v>0.1628083515364393</v>
+      </c>
+      <c r="HU20" t="n">
+        <v>0.08609891274509143</v>
+      </c>
+      <c r="HV20" t="n">
+        <v>0.248227066164654</v>
+      </c>
+      <c r="HW20" t="n">
+        <v>0.1708320907233919</v>
+      </c>
+      <c r="HX20" t="n">
+        <v>0.1652376664423863</v>
+      </c>
+      <c r="HY20" t="n">
+        <v>0.1714671200023311</v>
+      </c>
+      <c r="HZ20" t="n">
+        <v>0.167013324028484</v>
+      </c>
+      <c r="IA20" t="n">
+        <v>0.153563669574363</v>
+      </c>
+      <c r="IB20" t="n">
+        <v>0.242254021228352</v>
+      </c>
+      <c r="IC20" t="n">
+        <v>0.1628083515364393</v>
+      </c>
+      <c r="ID20" t="n">
+        <v>0.1779700841721669</v>
+      </c>
+      <c r="IE20" t="n">
+        <v>0.1630707866815285</v>
+      </c>
+      <c r="IF20" t="n">
+        <v>0.171149979304608</v>
+      </c>
+      <c r="IG20" t="n">
+        <v>0.1708320907233919</v>
+      </c>
+      <c r="IH20" t="n">
+        <v>0.1787639303337974</v>
+      </c>
+      <c r="II20" t="n">
+        <v>0.1898126509879515</v>
+      </c>
+      <c r="IJ20" t="n">
+        <v>0.153563669574363</v>
+      </c>
+      <c r="IK20" t="n">
+        <v>0.1656576508718449</v>
+      </c>
+      <c r="IL20" t="n">
+        <v>0.08527110065044263</v>
+      </c>
+      <c r="IM20" t="n">
+        <v>0.1016624231469964</v>
+      </c>
+      <c r="IN20" t="n">
+        <v>0.167013324028484</v>
+      </c>
+      <c r="IO20" t="n">
+        <v>0.1601042915911721</v>
+      </c>
+      <c r="IP20" t="n">
+        <v>0.1354999840670127</v>
+      </c>
+      <c r="IQ20" t="n">
+        <v>0.1223598759062027</v>
+      </c>
+      <c r="IR20" t="n">
+        <v>0.1787953692988891</v>
+      </c>
+      <c r="IS20" t="n">
+        <v>0.1766083512288195</v>
+      </c>
+      <c r="IT20" t="n">
+        <v>0.174642684074014</v>
+      </c>
+      <c r="IU20" t="n">
+        <v>0.2406482117432866</v>
+      </c>
+      <c r="IV20" t="n">
+        <v>0.1738473063614777</v>
+      </c>
+      <c r="IW20" t="n">
+        <v>0.1791621985574765</v>
+      </c>
+      <c r="IX20" t="n">
+        <v>0.2577715756711185</v>
+      </c>
+      <c r="IY20" t="n">
+        <v>0.2931007937738884</v>
+      </c>
+      <c r="IZ20" t="n">
+        <v>0.1425831385804173</v>
+      </c>
+      <c r="JA20" t="n">
+        <v>0.1477669394259286</v>
+      </c>
+      <c r="JB20" t="n">
+        <v>0.1436872365754285</v>
+      </c>
+      <c r="JC20" t="n">
+        <v>0.1421647899115296</v>
+      </c>
+      <c r="JD20" t="n">
+        <v>0.1638937448190528</v>
+      </c>
+      <c r="JE20" t="n">
+        <v>0.1553594958261904</v>
+      </c>
+      <c r="JF20" t="n">
+        <v>0.1564272921199261</v>
+      </c>
+      <c r="JG20" t="n">
+        <v>0.1647518217323552</v>
+      </c>
+      <c r="JH20" t="n">
+        <v>0.1498075128539083</v>
+      </c>
+      <c r="JI20" t="n">
+        <v>0.1582769952107441</v>
+      </c>
+      <c r="JJ20" t="n">
+        <v>0.1541141584725105</v>
+      </c>
+      <c r="JK20" t="n">
+        <v>0.1647689995508312</v>
+      </c>
+      <c r="JL20" t="n">
+        <v>0.1631212371597368</v>
+      </c>
+      <c r="JM20" t="n">
+        <v>0.164260759861625</v>
+      </c>
+      <c r="JN20" t="n">
+        <v>0.1780274845369086</v>
+      </c>
+      <c r="JO20" t="n">
+        <v>0.1673037202060231</v>
+      </c>
+      <c r="JP20" t="n">
+        <v>0.1814044858003223</v>
+      </c>
+      <c r="JQ20" t="n">
+        <v>0.1682181945093628</v>
       </c>
     </row>
   </sheetData>

</xml_diff>